<commit_message>
Update Register doc with cmd list formats
</commit_message>
<xml_diff>
--- a/rtl/user_domain/reg_address_map.xlsx
+++ b/rtl/user_domain/reg_address_map.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ecp\croc\rtl\user_domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{191E4983-81C2-4C8B-9883-B68A07E2F833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDC8B256-990D-424B-B70A-092AE912B8BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-9670" windowWidth="38620" windowHeight="21100" xr2:uid="{CCB46CB1-C430-44BE-A5E2-4295C43B14BB}"/>
   </bookViews>
   <sheets>
     <sheet name="ascom regs" sheetId="3" r:id="rId1"/>
-    <sheet name="State Diagrams" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="87">
   <si>
     <t>R</t>
   </si>
@@ -192,163 +191,112 @@
     <t>ASCON_MODE</t>
   </si>
   <si>
-    <t xml:space="preserve">    printf("Encode test\n");</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_CONTROL] = 0;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_KEY    ] = (long)key; // send a key before starting enc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    while( ( hw_reg[REG_STATUS] &amp; STATUS_KEY_DMA ) == 0  ); // wait for key data to start</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_MODE] = MODE_ENC; // put into encode mode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    while( ( hw_reg[REG_STATUS] &amp; STATUS_KEY_CMD ) == 0  ); // wait for key cmd complete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_LENGTH ] = 16 ; // set nonce length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_CONTROL] = BDI_EOT + BDI_TYPE_NONCE;  // set to 1 message nonce</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_BDI    ] = (long)npub; // send nonce via bdi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    while( ( hw_reg[REG_STATUS] &amp; STATUS_BDI_CMD ) == 0  ); // wait for nonce bdi to complete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_LENGTH ] = 9; // set ad length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_CONTROL] = BDI_EOT + BDI_TYPE_AD; // set to AS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_BDI    ] = (long)ad; // send ad via bdi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    while( ( hw_reg[REG_STATUS] &amp; STATUS_BDI_CMD ) == 0  ); // wait for bdi send</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_LENGTH ] = 9; // set msg length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_CONTROL] = BDI_LIO + BDI_EOT + BDI_EOI + BDI_TYPE_MSG; // Set to msg type, last input, link in-out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_BDO    ] = (long)pt; // start BDO write</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_BDI    ] = (long)pt; // start BDI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    while( ( hw_reg[REG_STATUS] &amp; STATUS_BDI_CMD ) == 0  ); // wait BDI complete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    while( ( hw_reg[REG_STATUS] &amp; STATUS_BDO_CMD ) == 0  ); // wait BDO complete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_CONTROL] = 0; // turn off LIO </t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_LENGTH ] = 16; // set tag length (128 bits fixed)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    hw_reg[REG_BDO    ] = (long)tag; // start BDO for tag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    while( ( hw_reg[REG_STATUS] &amp; STATUS_BDO_CMD ) == 0  ); // wait for BDO write complete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    while( ( hw_reg[REG_STATUS] &amp; STATUS_DONE ) == 0  ); // wait/confirm cipher is done</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    printf("Done\n");</t>
-  </si>
-  <si>
-    <t>WAIT_KEY_DONE</t>
-  </si>
-  <si>
-    <t>WAIT_KEY_DATA</t>
-  </si>
-  <si>
-    <t>MODE ENCODE</t>
-  </si>
-  <si>
-    <t>Column1</t>
-  </si>
-  <si>
-    <t>Column2</t>
-  </si>
-  <si>
-    <t>Column3</t>
-  </si>
-  <si>
-    <t>Column4</t>
-  </si>
-  <si>
-    <t>Column5</t>
-  </si>
-  <si>
-    <t>Column6</t>
-  </si>
-  <si>
-    <t>Column7</t>
-  </si>
-  <si>
-    <t>Column8</t>
-  </si>
-  <si>
-    <t>Column9</t>
-  </si>
-  <si>
-    <t>WAIT BDI DONE</t>
-  </si>
-  <si>
-    <t>WAIT CMD ADDR</t>
-  </si>
-  <si>
-    <t>WAIT BDO DONE</t>
-  </si>
-  <si>
-    <t>BDI_TYPE = MSG, EOI, EOT, LOI</t>
-  </si>
-  <si>
-    <t>BDI_TYPE = 0 // turn off LOI</t>
-  </si>
-  <si>
-    <t>WAIT ASCON DONE</t>
-  </si>
-  <si>
-    <t>SEND KEY (read_next(), 16)</t>
-  </si>
-  <si>
-    <t>LATCH ad_len, msg_len</t>
-  </si>
-  <si>
-    <t>SEND BDI (read_next(), 16) // nonce</t>
-  </si>
-  <si>
-    <t>SEND BDI (read_next, ad_len) // ad</t>
-  </si>
-  <si>
-    <t>RECV BDO(read_next, 16) // tag (signature)</t>
-  </si>
-  <si>
-    <t>BDI_TYPE = NONCE, EOT, EOI = ( ad_len==0 &amp;&amp; msg_len==0)</t>
-  </si>
-  <si>
-    <t>BDI_TYPE = AD, EOT, EOI = ( msg_len == 0 )</t>
-  </si>
-  <si>
-    <t>RECV BDO(read_next, ,sg_len) // msg ct</t>
-  </si>
-  <si>
-    <t>SEND BDI (read_next, msg_len) // msg pt</t>
+    <t>Loi</t>
+  </si>
+  <si>
+    <t>msg_len</t>
+  </si>
+  <si>
+    <t>modifier</t>
+  </si>
+  <si>
+    <t>ad_len</t>
+  </si>
+  <si>
+    <t>auth_valid</t>
+  </si>
+  <si>
+    <t>Encode</t>
+  </si>
+  <si>
+    <t>Deocde</t>
+  </si>
+  <si>
+    <t>Hash</t>
+  </si>
+  <si>
+    <t>Xof</t>
+  </si>
+  <si>
+    <t>Cxof</t>
+  </si>
+  <si>
+    <t>*key</t>
+  </si>
+  <si>
+    <t>*nonce</t>
+  </si>
+  <si>
+    <t>*ad</t>
+  </si>
+  <si>
+    <t>*tag</t>
+  </si>
+  <si>
+    <t>*tag(w)</t>
+  </si>
+  <si>
+    <t>*auth(w)</t>
+  </si>
+  <si>
+    <t>RW</t>
+  </si>
+  <si>
+    <t>*pt</t>
+  </si>
+  <si>
+    <t>*ct</t>
+  </si>
+  <si>
+    <t>*msg</t>
+  </si>
+  <si>
+    <t>*hash</t>
+  </si>
+  <si>
+    <t>hash_len</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>*ctsm</t>
+  </si>
+  <si>
+    <t>key[16]</t>
+  </si>
+  <si>
+    <t>nonce[16]</t>
+  </si>
+  <si>
+    <t>*vhash</t>
+  </si>
+  <si>
+    <t>ad[ad_len]</t>
+  </si>
+  <si>
+    <t>pt[msg_len]</t>
+  </si>
+  <si>
+    <t>tag[16];</t>
+  </si>
+  <si>
+    <t>auth[4]</t>
+  </si>
+  <si>
+    <t>msg[msg_len]</t>
+  </si>
+  <si>
+    <t>hash[32]</t>
+  </si>
+  <si>
+    <t>vhash[hash_len]</t>
+  </si>
+  <si>
+    <t>ctsm[ad_len]</t>
+  </si>
+  <si>
+    <t>CMD#</t>
   </si>
 </sst>
 </file>
@@ -371,14 +319,15 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -390,13 +339,8 @@
         <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="12">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -529,13 +473,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -611,10 +574,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" textRotation="45"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" textRotation="45"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Good" xfId="2" builtinId="26"/>
+  <cellStyles count="2">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -629,24 +607,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{352411B4-AC10-4687-8FBB-8E12CC2C98F0}" name="Table1" displayName="Table1" ref="B4:J34" totalsRowShown="0">
-  <autoFilter ref="B4:J34" xr:uid="{352411B4-AC10-4687-8FBB-8E12CC2C98F0}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{6EF46EA7-CD5F-4ADB-A4D6-50B0BA816CDC}" name="Column1"/>
-    <tableColumn id="2" xr3:uid="{E7123E65-A6DC-4933-AE27-AAEF1544F2E4}" name="Column2"/>
-    <tableColumn id="3" xr3:uid="{CEF05FA4-FD14-4862-9AFE-8CA39D817AA6}" name="Column3"/>
-    <tableColumn id="4" xr3:uid="{9F795AA5-3125-44F7-88C1-29F7E338C0AC}" name="Column4"/>
-    <tableColumn id="5" xr3:uid="{8E5306FF-4FDE-42A2-9DCD-77048D76DDC4}" name="Column5"/>
-    <tableColumn id="6" xr3:uid="{85EDF337-22A5-42A5-8820-B057CF467E32}" name="Column6"/>
-    <tableColumn id="7" xr3:uid="{A35395E3-0479-4DE0-917D-BFA3F745E486}" name="Column7"/>
-    <tableColumn id="8" xr3:uid="{5E3F9508-56E7-4EB8-AC77-55364EB1A655}" name="Column8"/>
-    <tableColumn id="9" xr3:uid="{E4293814-B054-4AA7-BA05-500586688C15}" name="Column9"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -946,13 +906,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{738A60D2-D720-4AFC-80B7-9351B49089D5}">
-  <dimension ref="B3:AJ19"/>
+  <dimension ref="B3:AJ32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="15.81640625" customWidth="1"/>
     <col min="3" max="4" width="8.7265625" style="1"/>
     <col min="5" max="5" width="5.54296875" customWidth="1"/>
-    <col min="6" max="23" width="2.81640625" customWidth="1"/>
+    <col min="6" max="7" width="2.81640625" customWidth="1"/>
+    <col min="8" max="8" width="2.90625" customWidth="1"/>
+    <col min="9" max="9" width="4.26953125" customWidth="1"/>
+    <col min="10" max="23" width="2.81640625" customWidth="1"/>
     <col min="24" max="24" width="3.7265625" customWidth="1"/>
     <col min="25" max="30" width="2.81640625" customWidth="1"/>
     <col min="31" max="31" width="4.6328125" customWidth="1"/>
@@ -1459,7 +1422,7 @@
       <c r="AI12" s="16"/>
       <c r="AJ12" s="18"/>
     </row>
-    <row r="13" spans="2:36" ht="46" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>3</v>
       </c>
@@ -1475,7 +1438,9 @@
       <c r="F13" s="16"/>
       <c r="G13" s="17"/>
       <c r="H13" s="26"/>
-      <c r="I13" s="10"/>
+      <c r="I13" s="6" t="s">
+        <v>55</v>
+      </c>
       <c r="J13" s="6" t="s">
         <v>29</v>
       </c>
@@ -1745,6 +1710,9 @@
       <c r="W18" s="3"/>
       <c r="X18" s="5" t="s">
         <v>4</v>
+      </c>
+      <c r="AB18" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="AC18" s="3"/>
       <c r="AD18" s="3"/>
@@ -1806,250 +1774,428 @@
       <c r="AI19" s="3"/>
       <c r="AJ19" s="4"/>
     </row>
+    <row r="22" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="D22" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="23" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="D23" s="1">
+        <v>0</v>
+      </c>
+      <c r="E23" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="33"/>
+      <c r="I23" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="J23" s="32"/>
+      <c r="K23" s="32"/>
+      <c r="L23" s="33"/>
+      <c r="M23" s="9"/>
+      <c r="N23" s="41"/>
+      <c r="O23" s="41"/>
+      <c r="P23" s="41"/>
+      <c r="Q23" s="41"/>
+      <c r="R23" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="S23" s="32"/>
+      <c r="T23" s="32"/>
+      <c r="U23" s="32"/>
+      <c r="V23" s="32"/>
+      <c r="W23" s="32"/>
+      <c r="X23" s="33"/>
+      <c r="Y23" s="2"/>
+      <c r="Z23" s="3"/>
+      <c r="AA23" s="3"/>
+      <c r="AB23" s="3"/>
+      <c r="AC23" s="3"/>
+      <c r="AD23" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AE23" s="19"/>
+      <c r="AF23" s="19"/>
+      <c r="AG23" s="20"/>
+      <c r="AH23" s="16"/>
+      <c r="AI23" s="16"/>
+      <c r="AJ23" s="18"/>
+    </row>
+    <row r="24" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="16"/>
+      <c r="N24" s="16"/>
+      <c r="O24" s="16"/>
+      <c r="P24" s="16"/>
+      <c r="Q24" s="16"/>
+      <c r="R24" s="3"/>
+      <c r="S24" s="3"/>
+      <c r="T24" s="3"/>
+      <c r="U24" s="3"/>
+      <c r="V24" s="3"/>
+      <c r="W24" s="3"/>
+      <c r="X24" s="3"/>
+      <c r="Y24" s="29"/>
+      <c r="Z24" s="29"/>
+      <c r="AA24" s="29"/>
+      <c r="AB24" s="29"/>
+      <c r="AC24" s="29"/>
+      <c r="AD24" s="29"/>
+      <c r="AE24" s="21"/>
+      <c r="AF24" s="21"/>
+      <c r="AG24" s="22"/>
+      <c r="AH24" s="30"/>
+      <c r="AI24" s="30"/>
+      <c r="AJ24" s="30"/>
+    </row>
+    <row r="25" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="E25" s="37">
+        <v>1</v>
+      </c>
+      <c r="F25" s="29"/>
+      <c r="G25" s="29"/>
+      <c r="H25" s="38"/>
+      <c r="I25" s="37">
+        <v>2</v>
+      </c>
+      <c r="J25" s="29"/>
+      <c r="K25" s="29"/>
+      <c r="L25" s="38"/>
+      <c r="M25" s="37">
+        <v>3</v>
+      </c>
+      <c r="N25" s="29"/>
+      <c r="O25" s="29"/>
+      <c r="P25" s="38"/>
+      <c r="Q25" s="37">
+        <v>4</v>
+      </c>
+      <c r="R25" s="29"/>
+      <c r="S25" s="29"/>
+      <c r="T25" s="38"/>
+      <c r="U25" s="37">
+        <v>5</v>
+      </c>
+      <c r="V25" s="29"/>
+      <c r="W25" s="29"/>
+      <c r="X25" s="38"/>
+      <c r="Y25" s="29"/>
+      <c r="Z25" s="29"/>
+      <c r="AA25" s="29"/>
+      <c r="AB25" s="29"/>
+      <c r="AC25" s="29"/>
+      <c r="AD25" s="29"/>
+      <c r="AE25" s="21"/>
+      <c r="AF25" s="21"/>
+      <c r="AG25" s="22"/>
+      <c r="AH25" s="30"/>
+      <c r="AI25" s="30"/>
+      <c r="AJ25" s="30"/>
+    </row>
+    <row r="26" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="E26" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="F26" s="35"/>
+      <c r="G26" s="35"/>
+      <c r="H26" s="36"/>
+      <c r="I26" s="34" t="s">
+        <v>57</v>
+      </c>
+      <c r="J26" s="35"/>
+      <c r="K26" s="35"/>
+      <c r="L26" s="36"/>
+      <c r="M26" s="34" t="s">
+        <v>58</v>
+      </c>
+      <c r="N26" s="35"/>
+      <c r="O26" s="35"/>
+      <c r="P26" s="36"/>
+      <c r="Q26" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="R26" s="35"/>
+      <c r="S26" s="35"/>
+      <c r="T26" s="36"/>
+      <c r="U26" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="V26" s="35"/>
+      <c r="W26" s="29"/>
+      <c r="X26" s="38"/>
+      <c r="AC26" t="s">
+        <v>75</v>
+      </c>
+      <c r="AG26" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="27" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="D27" s="1">
+        <v>1</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="F27" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="G27" s="29"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="J27" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="K27" s="29"/>
+      <c r="L27" s="38"/>
+      <c r="M27" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="N27" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="O27" s="29"/>
+      <c r="P27" s="38"/>
+      <c r="Q27" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="R27" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="S27" s="29"/>
+      <c r="T27" s="38"/>
+      <c r="U27" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="V27" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="W27" s="29"/>
+      <c r="X27" s="38"/>
+      <c r="AC27" t="s">
+        <v>76</v>
+      </c>
+      <c r="AG27" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="28" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="D28" s="1">
+        <v>2</v>
+      </c>
+      <c r="E28" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="F28" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="G28" s="29"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="J28" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="K28" s="29"/>
+      <c r="L28" s="38"/>
+      <c r="M28" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="N28" s="29" t="s">
+        <v>71</v>
+      </c>
+      <c r="O28" s="29"/>
+      <c r="P28" s="38"/>
+      <c r="Q28" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="R28" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="S28" s="29"/>
+      <c r="T28" s="38"/>
+      <c r="U28" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="V28" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="W28" s="29"/>
+      <c r="X28" s="38"/>
+      <c r="AC28" t="s">
+        <v>78</v>
+      </c>
+      <c r="AG28" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="29" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="D29" s="1">
+        <v>3</v>
+      </c>
+      <c r="E29" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="F29" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="G29" s="29"/>
+      <c r="H29" s="38"/>
+      <c r="I29" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="J29" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="K29" s="29"/>
+      <c r="L29" s="38"/>
+      <c r="M29" s="37"/>
+      <c r="N29" s="29"/>
+      <c r="O29" s="29"/>
+      <c r="P29" s="38"/>
+      <c r="Q29" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="R29" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="S29" s="29"/>
+      <c r="T29" s="38"/>
+      <c r="U29" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="V29" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="W29" s="29"/>
+      <c r="X29" s="38"/>
+      <c r="AC29" t="s">
+        <v>79</v>
+      </c>
+      <c r="AG29" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="30" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="D30" s="1">
+        <v>4</v>
+      </c>
+      <c r="E30" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="F30" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="G30" s="29"/>
+      <c r="H30" s="38"/>
+      <c r="I30" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="J30" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="K30" s="29"/>
+      <c r="L30" s="38"/>
+      <c r="M30" s="37"/>
+      <c r="N30" s="29"/>
+      <c r="O30" s="29"/>
+      <c r="P30" s="38"/>
+      <c r="Q30" s="37"/>
+      <c r="R30" s="29"/>
+      <c r="S30" s="29"/>
+      <c r="T30" s="38"/>
+      <c r="U30" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="V30" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="W30" s="29"/>
+      <c r="X30" s="38"/>
+      <c r="AC30" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="D31" s="1">
+        <v>5</v>
+      </c>
+      <c r="E31" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F31" s="29" t="s">
+        <v>65</v>
+      </c>
+      <c r="G31" s="29"/>
+      <c r="H31" s="38"/>
+      <c r="I31" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="J31" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="K31" s="29"/>
+      <c r="L31" s="38"/>
+      <c r="M31" s="37"/>
+      <c r="N31" s="29"/>
+      <c r="O31" s="29"/>
+      <c r="P31" s="38"/>
+      <c r="Q31" s="37"/>
+      <c r="R31" s="29"/>
+      <c r="S31" s="29"/>
+      <c r="T31" s="38"/>
+      <c r="U31" s="37"/>
+      <c r="V31" s="29"/>
+      <c r="W31" s="29"/>
+      <c r="X31" s="38"/>
+      <c r="AC31" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="32" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="D32" s="1">
+        <v>6</v>
+      </c>
+      <c r="E32" s="39"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="40"/>
+      <c r="I32" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="J32" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="K32" s="27"/>
+      <c r="L32" s="40"/>
+      <c r="M32" s="39"/>
+      <c r="N32" s="27"/>
+      <c r="O32" s="27"/>
+      <c r="P32" s="40"/>
+      <c r="Q32" s="39"/>
+      <c r="R32" s="27"/>
+      <c r="S32" s="27"/>
+      <c r="T32" s="40"/>
+      <c r="U32" s="39"/>
+      <c r="V32" s="27"/>
+      <c r="W32" s="27"/>
+      <c r="X32" s="40"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2392D002-1580-4B7D-B92D-915D0C8A379C}">
-  <dimension ref="B4:J34"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="99.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="10" width="9" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E4" t="s">
-        <v>83</v>
-      </c>
-      <c r="F4" t="s">
-        <v>84</v>
-      </c>
-      <c r="G4" t="s">
-        <v>85</v>
-      </c>
-      <c r="H4" t="s">
-        <v>86</v>
-      </c>
-      <c r="I4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="D7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
-        <v>53</v>
-      </c>
-      <c r="D11" s="29" t="s">
-        <v>95</v>
-      </c>
-      <c r="E11" s="29"/>
-    </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B12" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B13" t="s">
-        <v>55</v>
-      </c>
-      <c r="D13" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B14" t="s">
-        <v>56</v>
-      </c>
-      <c r="D14" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B15" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B16" t="s">
-        <v>58</v>
-      </c>
-      <c r="D16" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B17" t="s">
-        <v>59</v>
-      </c>
-      <c r="D17" s="29" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" t="s">
-        <v>60</v>
-      </c>
-      <c r="D18" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" t="s">
-        <v>62</v>
-      </c>
-      <c r="D20" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" t="s">
-        <v>63</v>
-      </c>
-      <c r="D21" s="29" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B22" t="s">
-        <v>64</v>
-      </c>
-      <c r="D22" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B23" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B24" t="s">
-        <v>66</v>
-      </c>
-      <c r="D24" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D25" s="29" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B26" t="s">
-        <v>68</v>
-      </c>
-      <c r="D26" s="29" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B27" t="s">
-        <v>69</v>
-      </c>
-      <c r="D27" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B28" t="s">
-        <v>70</v>
-      </c>
-      <c r="D28" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B29" t="s">
-        <v>71</v>
-      </c>
-      <c r="D29" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B30" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B31" t="s">
-        <v>73</v>
-      </c>
-      <c r="D31" s="29" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B32" t="s">
-        <v>74</v>
-      </c>
-      <c r="D32" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B33" t="s">
-        <v>75</v>
-      </c>
-      <c r="D33" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B34" t="s">
-        <v>76</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>